<commit_message>
delete of useless plots
</commit_message>
<xml_diff>
--- a/Data/claim_firm_sep.xlsx
+++ b/Data/claim_firm_sep.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcel/Documents/GitHub/Stage_BxSE/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F528055C-58F5-0541-BBE0-36834F8F9D08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD67A955-9A7D-6645-8DCD-5F273507B000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="51">
   <si>
     <t>Claimants</t>
   </si>
@@ -173,6 +173,9 @@
   </si>
   <si>
     <t>Own Repot</t>
+  </si>
+  <si>
+    <t>Category</t>
   </si>
 </sst>
 </file>
@@ -532,7 +535,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="48.33203125" bestFit="1" customWidth="1"/>
@@ -542,7 +545,7 @@
     <col min="8" max="8" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -567,8 +570,11 @@
       <c r="H1" s="1" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I1" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -594,7 +600,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -608,7 +614,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -622,7 +628,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -636,7 +642,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -650,7 +656,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
@@ -664,7 +670,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -690,7 +696,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -716,7 +722,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -730,7 +736,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -744,7 +750,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -770,7 +776,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>18</v>
       </c>
@@ -796,7 +802,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -822,7 +828,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -848,7 +854,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>20</v>
       </c>

</xml_diff>